<commit_message>
Refine subtyping comparison reports
</commit_message>
<xml_diff>
--- a/HCVData/subtyping-comparison-all-ras/12-report-subtype-disagreements/Subtype_Disagreement_Reports.xlsx
+++ b/HCVData/subtyping-comparison-all-ras/12-report-subtype-disagreements/Subtype_Disagreement_Reports.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="188">
   <si>
     <t>CometSubtype</t>
   </si>
@@ -41,577 +41,550 @@
     <t>1A</t>
   </si>
   <si>
-    <t>86</t>
+    <t>87</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>106</t>
+  </si>
+  <si>
+    <t>1A;1B;1C;1J;1K;1M;1N;1O;1P;3A</t>
+  </si>
+  <si>
+    <t>1B</t>
+  </si>
+  <si>
+    <t>105</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>115</t>
+  </si>
+  <si>
+    <t>1A;1B;1C;1D;1H;1I;1K;1M;1N;1O;2L;3A;6D;6P;6XD;6XF;6XG;7B</t>
+  </si>
+  <si>
+    <t>1C</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1A;1C;1O</t>
+  </si>
+  <si>
+    <t>1E</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1A;1E</t>
+  </si>
+  <si>
+    <t>1G</t>
+  </si>
+  <si>
+    <t>1B;1G</t>
+  </si>
+  <si>
+    <t>1H</t>
+  </si>
+  <si>
+    <t>1B;1C;1H</t>
+  </si>
+  <si>
+    <t>1L</t>
+  </si>
+  <si>
+    <t>1B;1L</t>
+  </si>
+  <si>
+    <t>2A</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>2A;2M;2Q;2R;2U</t>
+  </si>
+  <si>
+    <t>2B</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>2B;2C;2L;2Q;2T</t>
+  </si>
+  <si>
+    <t>2C</t>
+  </si>
+  <si>
+    <t>2C;2F;2Q</t>
+  </si>
+  <si>
+    <t>2J</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>2A;2C;2D;2E;2F;2I;2J;2M;2Q;2R;2T;2U;2V;5A;7A</t>
+  </si>
+  <si>
+    <t>2K</t>
+  </si>
+  <si>
+    <t>2D;2J;2K;2Q</t>
+  </si>
+  <si>
+    <t>2Q</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>2K;2Q</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>1A;1B;3A;3D;3E</t>
+  </si>
+  <si>
+    <t>3G</t>
+  </si>
+  <si>
+    <t>3B;3G;3I</t>
+  </si>
+  <si>
+    <t>3H</t>
+  </si>
+  <si>
+    <t>3H;8A</t>
+  </si>
+  <si>
+    <t>4A</t>
+  </si>
+  <si>
+    <t>4A;4C;4E;4P</t>
+  </si>
+  <si>
+    <t>4F</t>
+  </si>
+  <si>
+    <t>4C;4E;4F;4Q</t>
+  </si>
+  <si>
+    <t>4K</t>
+  </si>
+  <si>
+    <t>4B;4G;4H;4K;4R;6Q</t>
+  </si>
+  <si>
+    <t>4L</t>
+  </si>
+  <si>
+    <t>4L;4V</t>
+  </si>
+  <si>
+    <t>4M</t>
+  </si>
+  <si>
+    <t>1B;4M</t>
+  </si>
+  <si>
+    <t>4R</t>
+  </si>
+  <si>
+    <t>4A;4R</t>
+  </si>
+  <si>
+    <t>4V</t>
+  </si>
+  <si>
+    <t>4B;4Q;4V</t>
+  </si>
+  <si>
+    <t>4W</t>
+  </si>
+  <si>
+    <t>4B;4W</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>6A</t>
+  </si>
+  <si>
+    <t>6A;6B;6XD</t>
+  </si>
+  <si>
+    <t>6C</t>
+  </si>
+  <si>
+    <t>1H;6C</t>
+  </si>
+  <si>
+    <t>6D</t>
+  </si>
+  <si>
+    <t>1H;6D;8A</t>
+  </si>
+  <si>
+    <t>6E</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>1B;1C;6C;6E;6Q;6U;6XC;6XF;8A</t>
+  </si>
+  <si>
+    <t>6G</t>
+  </si>
+  <si>
+    <t>6K</t>
+  </si>
+  <si>
+    <t>6K;6K-RELATED;6XI;8A</t>
+  </si>
+  <si>
+    <t>6L</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>1A;6K;6K-RELATED;6L;6L-RELATED;6XB;6XI;6XJ;8A</t>
+  </si>
+  <si>
+    <t>6M</t>
+  </si>
+  <si>
+    <t>6M;8A</t>
+  </si>
+  <si>
+    <t>6N</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>6N;6XE;6XG</t>
+  </si>
+  <si>
+    <t>6O</t>
+  </si>
+  <si>
+    <t>6O;6Q</t>
+  </si>
+  <si>
+    <t>6R</t>
+  </si>
+  <si>
+    <t>1K;6R</t>
+  </si>
+  <si>
+    <t>6W</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>6A;6D;6G;6H;6L;6N;6Q;6S;6W;6XA;6XD;6XF;6XH;8A</t>
+  </si>
+  <si>
+    <t>6XA</t>
+  </si>
+  <si>
+    <t>6U;6XA</t>
+  </si>
+  <si>
+    <t>7A</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 1A-1B</t>
+  </si>
+  <si>
+    <t>1A;1B;UNASSIGNED_1, 1A-1B</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 1B-1A</t>
+  </si>
+  <si>
+    <t>1A;1B;1I;UNASSIGNED_1, 1B-1A</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 1B-6W</t>
+  </si>
+  <si>
+    <t>8A;UNASSIGNED_1, 1B-6W</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 2J-5A</t>
+  </si>
+  <si>
+    <t>8A;UNASSIGNED_1, 2J-5A</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 4D-4O</t>
+  </si>
+  <si>
+    <t>4D;UNASSIGNED_1, 4D-4O</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 4V-4G</t>
+  </si>
+  <si>
+    <t>4S;UNASSIGNED_1, 4V-4G</t>
+  </si>
+  <si>
+    <t>UNASSIGNED_1, 5A-1C</t>
+  </si>
+  <si>
+    <t>5B;UNASSIGNED_1, 5A-1C</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>1A;1B;1C;1D;1G;1H;1I;1K;1L;1M;1N;1O;2K;5A;6B;6D;6P;6U;6W;6XA;6XD;6XG</t>
+  </si>
+  <si>
+    <t>1C;1E;1N;1O</t>
+  </si>
+  <si>
+    <t>1D;1H</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>1A;1B;1J;1K;1M;1N;3A</t>
-  </si>
-  <si>
-    <t>1B</t>
-  </si>
-  <si>
-    <t>105</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>149</t>
-  </si>
-  <si>
-    <t>1A;1B;1C;1D;1H;1I;1K;1M;1N;1O;1P;2J;3A;5A;6D;6E;6G;6N;6P;6S;6W;6XA;6XD;6XF;6XG;6XH;7A;7B;8A;UNASSIGNED_1, 1A-1B;UNASSIGNED_1, 1B-1A;UNASSIGNED_1, 1B-6W;UNASSIGNED_1, 2J-5A</t>
-  </si>
-  <si>
-    <t>1C</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>1A;1C;1M;1O</t>
-  </si>
-  <si>
-    <t>1E</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>1A;1E</t>
-  </si>
-  <si>
-    <t>1G</t>
-  </si>
-  <si>
-    <t>1B;1G</t>
-  </si>
-  <si>
-    <t>1H</t>
-  </si>
-  <si>
-    <t>1B;1C;1H</t>
-  </si>
-  <si>
-    <t>1L</t>
-  </si>
-  <si>
-    <t>1B;1L</t>
-  </si>
-  <si>
-    <t>2A</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>2A;2J;2M;2Q;2U;2V;7A</t>
-  </si>
-  <si>
-    <t>2B</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>2B;2C;2D;2J;2L;2M;2Q;2T;5A;5B;6A;6G;6W;6XA;6XD;6XH;8A;UNASSIGNED_1, 5A-1C</t>
-  </si>
-  <si>
-    <t>2C</t>
-  </si>
-  <si>
-    <t>1B;2C;2F;2J;2L;2Q;2R</t>
-  </si>
-  <si>
-    <t>2J</t>
+    <t>2A;2C;2F;2M;2P;2Q;2R;2U</t>
+  </si>
+  <si>
+    <t>2B;2E;2L;2Q;2T;7B</t>
+  </si>
+  <si>
+    <t>2B;2C;2F;2O</t>
+  </si>
+  <si>
+    <t>9</t>
   </si>
   <si>
     <t>24</t>
   </si>
   <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>2A;2C;2D;2E;2F;2I;2J;2K;2M;2Q;2R;2T;2U;2V;6E;6Q</t>
-  </si>
-  <si>
-    <t>2K</t>
+    <t>33</t>
+  </si>
+  <si>
+    <t>2A;2C;2D;2E;2F;2I;2J;2M;2Q;2R;2U;2V</t>
+  </si>
+  <si>
+    <t>2F;2K;2Q;2U</t>
+  </si>
+  <si>
+    <t>2A;2K;2Q;2R;2U</t>
+  </si>
+  <si>
+    <t>1A;3A;3B;3D;3E;7B</t>
+  </si>
+  <si>
+    <t>3G;3I</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>4A;4C;4E;4L;4N;4R;4V</t>
+  </si>
+  <si>
+    <t>4D</t>
+  </si>
+  <si>
+    <t>1A;1D;4A;4D</t>
+  </si>
+  <si>
+    <t>4C;4E;4F;4G;4V</t>
+  </si>
+  <si>
+    <t>1E;4A;4B;4D;4G;4H;4K;4L;4R;4V</t>
+  </si>
+  <si>
+    <t>4O</t>
+  </si>
+  <si>
+    <t>4O;4P;4V</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>2A;2D;2J;2K;2M;2Q;2R</t>
-  </si>
-  <si>
-    <t>2M</t>
-  </si>
-  <si>
-    <t>2J;2M;2Q</t>
-  </si>
-  <si>
-    <t>2Q</t>
-  </si>
-  <si>
-    <t>2A;2M;2Q</t>
-  </si>
-  <si>
-    <t>3A</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>1A;1B;3A;3D;3E</t>
+    <t>1A;1B;1K;4R</t>
+  </si>
+  <si>
+    <t>4L;4M;4O;4P;4Q;4V</t>
+  </si>
+  <si>
+    <t>1C;4V;6C;6E;6P;6Q;6XC;6XF;8A</t>
+  </si>
+  <si>
+    <t>5A;5B;6G</t>
+  </si>
+  <si>
+    <t>6J</t>
+  </si>
+  <si>
+    <t>6K;6K-RELATED;6L;6L-RELATED;6XB;6XI;6XJ;8A</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>4C;4D;4V;5A;6N;6XE;6XG</t>
+  </si>
+  <si>
+    <t>6T</t>
+  </si>
+  <si>
+    <t>4R;6T</t>
+  </si>
+  <si>
+    <t>5A;6G;6H;6L;6N;6Q;6T;6V;6W;6XA;6XE;6XF;6XG;6XH;8A</t>
+  </si>
+  <si>
+    <t>1D;5A;6U;6XA</t>
+  </si>
+  <si>
+    <t>1A;1I;UNASSIGNED_1, 1A-1B</t>
+  </si>
+  <si>
+    <t>1A;1B;UNASSIGNED_1, 1B-1A</t>
+  </si>
+  <si>
+    <t>1A;1B;1C;1H;1J;1K;1M;1N;1O;1P;3A</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>1A;1B;1B-BASAL;1D;1E;1I;1K;1N;1O;2K;6D;6G;6O;6P;6R;6XD</t>
+  </si>
+  <si>
+    <t>1C;1O</t>
+  </si>
+  <si>
+    <t>2A;2L;2U</t>
+  </si>
+  <si>
+    <t>2B;2F;2V;7B</t>
+  </si>
+  <si>
+    <t>2C;2O;2V</t>
+  </si>
+  <si>
+    <t>2A;2C;2D;2F;2J;2K;2L;2P;2R;2U;2V;5A;7A;7B</t>
+  </si>
+  <si>
+    <t>1A;3A;3D;3E</t>
   </si>
   <si>
     <t>3B</t>
   </si>
   <si>
-    <t>3B;3G;3I</t>
-  </si>
-  <si>
-    <t>3H</t>
-  </si>
-  <si>
-    <t>3H;8A</t>
-  </si>
-  <si>
-    <t>4A</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>4A;4B;4C;4E;4F;4K;4P</t>
-  </si>
-  <si>
-    <t>4D</t>
-  </si>
-  <si>
-    <t>4D;UNASSIGNED_1, 4D-4O</t>
-  </si>
-  <si>
-    <t>4F</t>
-  </si>
-  <si>
-    <t>4F;4Q;4S;4V;6L;6W;6XD;UNASSIGNED_1, 4V-4G</t>
-  </si>
-  <si>
-    <t>4K</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>4B;4G;4H;4K;4R;6Q</t>
-  </si>
-  <si>
-    <t>4L</t>
-  </si>
-  <si>
-    <t>4L;4V</t>
-  </si>
-  <si>
-    <t>4M</t>
-  </si>
-  <si>
-    <t>1B;4M</t>
-  </si>
-  <si>
-    <t>4R</t>
-  </si>
-  <si>
-    <t>4A;4R</t>
-  </si>
-  <si>
-    <t>4V</t>
-  </si>
-  <si>
-    <t>4B;4Q;4V</t>
-  </si>
-  <si>
-    <t>4W</t>
-  </si>
-  <si>
-    <t>4B;4W</t>
-  </si>
-  <si>
-    <t>6A</t>
-  </si>
-  <si>
-    <t>6A;6B;6G;6XD</t>
-  </si>
-  <si>
-    <t>6C</t>
-  </si>
-  <si>
-    <t>1H;6C</t>
-  </si>
-  <si>
-    <t>6D</t>
-  </si>
-  <si>
-    <t>1H;6D;8A</t>
-  </si>
-  <si>
-    <t>6E</t>
-  </si>
-  <si>
-    <t>1B;1C;6C;6E;6Q;6U;6W;6XC;6XF</t>
-  </si>
-  <si>
-    <t>6L</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>1A;6K;6K-RELATED;6L;6L-RELATED;6XB;6XI;6XJ;8A</t>
-  </si>
-  <si>
-    <t>6M</t>
-  </si>
-  <si>
-    <t>6M;8A</t>
-  </si>
-  <si>
-    <t>6N</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>6N;6XE;6XG</t>
-  </si>
-  <si>
-    <t>6O</t>
-  </si>
-  <si>
-    <t>6C;6E</t>
-  </si>
-  <si>
-    <t>6R</t>
-  </si>
-  <si>
-    <t>1K;6R</t>
-  </si>
-  <si>
-    <t>6T</t>
-  </si>
-  <si>
-    <t>6E;6O;6Q</t>
-  </si>
-  <si>
-    <t>6W</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>6E;6G;6H;6L;6Q;6S;6W;6XA;6XF;6XH;6XJ;8A</t>
-  </si>
-  <si>
-    <t>6XA</t>
-  </si>
-  <si>
-    <t>6U;6XA</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>1A;1B;1C;1J;1K;1M;1N;1O;1P;3A;UNASSIGNED_1, 1A-1B;UNASSIGNED_1, 1B-1A</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>1A;1B;1C;1D;1G;1H;1I;1K;1L;1M;1N;1O;2K;5A;6G;6H;6Q;6T;6V;6W;6XA;6XE;6XF;6XG;UNASSIGNED_1, 1B-1A</t>
-  </si>
-  <si>
-    <t>1C;1E;1N;1O</t>
-  </si>
-  <si>
-    <t>1D;1H</t>
-  </si>
-  <si>
-    <t>6G;6Q;6W;6XG</t>
-  </si>
-  <si>
-    <t>2A;2B;2C;2F;2J;2L;2M;2P;2Q;2R;2U</t>
-  </si>
-  <si>
-    <t>1B;2B;2E;2Q;2T;6B;6D</t>
-  </si>
-  <si>
-    <t>2B;2C;2F;2O</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>2A;2B;2C;2D;2E;2F;2I;2J;2K;2L;2M;2Q;2R;2U;2V;6W;7A;8A;UNASSIGNED_1, 2J-5A</t>
-  </si>
-  <si>
-    <t>2F;2K;2U</t>
-  </si>
-  <si>
-    <t>2A;2C;2J;2K;2Q;2R;2U</t>
-  </si>
-  <si>
-    <t>1A;2B;3A;3B;3D;3E;6N;6W;6XA;7B;8A;UNASSIGNED_1, 2J-5A</t>
-  </si>
-  <si>
-    <t>3G</t>
-  </si>
-  <si>
-    <t>3G;3I</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>63</t>
-  </si>
-  <si>
-    <t>4A;4B;4C;4K;4L;4N;4R;4V;6E;6P;8A;UNASSIGNED_1, 1B-6W</t>
-  </si>
-  <si>
-    <t>4C</t>
-  </si>
-  <si>
-    <t>4A;4C</t>
-  </si>
-  <si>
-    <t>1A;1D;4A;4B;4D;4K;UNASSIGNED_1, 4D-4O</t>
-  </si>
-  <si>
-    <t>4F;4G</t>
-  </si>
-  <si>
-    <t>4G</t>
-  </si>
-  <si>
-    <t>4G;4H;4K</t>
-  </si>
-  <si>
-    <t>1B;1E;1H;4A;4D;4G;4H;4K;4L;4R;6D;6G;6L;6W;6XA;6XD;6XJ</t>
-  </si>
-  <si>
-    <t>5A;6W;8A</t>
-  </si>
-  <si>
-    <t>4O</t>
-  </si>
-  <si>
-    <t>4O;4P;4V</t>
+    <t>2F;3B</t>
+  </si>
+  <si>
+    <t>4A;4C;4D;4E</t>
+  </si>
+  <si>
+    <t>4C;4E;4F</t>
+  </si>
+  <si>
+    <t>4B;4G;4K</t>
   </si>
   <si>
     <t>4Q</t>
   </si>
   <si>
-    <t>4Q;4V</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>1A;1B;1K;4R;6E;6XF</t>
-  </si>
-  <si>
-    <t>4A;4C;4E;4F;4G;4K;4L;4M;4O;4P;4Q;4S;4V;UNASSIGNED_1, 4V-4G</t>
-  </si>
-  <si>
-    <t>5A</t>
-  </si>
-  <si>
-    <t>5B;UNASSIGNED_1, 5A-1C</t>
-  </si>
-  <si>
-    <t>1C;6A;6B;6E;6Q;6XC;6XD</t>
-  </si>
-  <si>
-    <t>6D;8A</t>
-  </si>
-  <si>
-    <t>4V;6E;6XC</t>
-  </si>
-  <si>
-    <t>6G</t>
-  </si>
-  <si>
-    <t>5B;6G</t>
-  </si>
-  <si>
-    <t>6I</t>
-  </si>
-  <si>
-    <t>6J</t>
-  </si>
-  <si>
-    <t>6K</t>
-  </si>
-  <si>
-    <t>6K;6K-RELATED;6L;6XI;6XJ;8A</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>6K;6K-RELATED;6L;6L-RELATED;6XB;6XI;6XJ;8A</t>
-  </si>
-  <si>
-    <t>4C;4D;4V;5A;6N;6XE;6XG</t>
-  </si>
-  <si>
-    <t>6C;6E;6K;6K-RELATED;6L;6Q;6XB</t>
-  </si>
-  <si>
-    <t>6Q</t>
-  </si>
-  <si>
-    <t>6E;6Q</t>
-  </si>
-  <si>
-    <t>4R;6E;6G;6Q;6T;6W</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>1B;5A;6G;6L;6O;6P;6Q;6U;6W;6XA;6XE;6XF;6XH;8A</t>
-  </si>
-  <si>
-    <t>1D;5A;6U;6XA</t>
-  </si>
-  <si>
-    <t>UNASSIGNED_1, 1A-1B</t>
-  </si>
-  <si>
-    <t>1A;1I;UNASSIGNED_1, 1A-1B</t>
-  </si>
-  <si>
-    <t>15</t>
+    <t>4P;4Q;4V</t>
+  </si>
+  <si>
+    <t>6A;6B;6P;6XD</t>
+  </si>
+  <si>
+    <t>6C;6E;6Q;6XC;6XF;8A</t>
+  </si>
+  <si>
+    <t>6H</t>
+  </si>
+  <si>
+    <t>6H;8A</t>
+  </si>
+  <si>
+    <t>1A;1G;6N;6XE;6XG;8A</t>
+  </si>
+  <si>
+    <t>6S</t>
+  </si>
+  <si>
+    <t>1J;6S</t>
   </si>
   <si>
     <t>37</t>
   </si>
   <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>1A;1B;1B-BASAL;1C;1D;1E;1H;1I;1K;1N;1O;1P;2K;UNASSIGNED_1, 1A-1B;UNASSIGNED_1, 1B-1A</t>
-  </si>
-  <si>
-    <t>1A;1C;1O</t>
-  </si>
-  <si>
-    <t>2A;2L;2U</t>
-  </si>
-  <si>
-    <t>2B;2F;2V;7B;8A;UNASSIGNED_1, 1B-6W</t>
-  </si>
-  <si>
-    <t>2C;2O;2V</t>
-  </si>
-  <si>
-    <t>2A;2C;2D;2F;2J;2K;2L;2P;2R;2U;2V</t>
-  </si>
-  <si>
-    <t>1A;3A;3D;3E;6W;8A</t>
-  </si>
-  <si>
-    <t>2F;3B</t>
-  </si>
-  <si>
-    <t>2J;4A;4C;4D;4P;4Q;4V;7B</t>
-  </si>
-  <si>
-    <t>4C;4E;4F</t>
-  </si>
-  <si>
-    <t>1B;4B;4G;4K;6R;6XD</t>
-  </si>
-  <si>
-    <t>4A;4B;4C;4E;4K;4Q;4S;4V;UNASSIGNED_1, 4V-4G</t>
-  </si>
-  <si>
-    <t>2J;5A;5B;UNASSIGNED_1, 5A-1C</t>
-  </si>
-  <si>
-    <t>2J;6A;6B;6R;6W;6XA;6XD;7A;8A;UNASSIGNED_1, 2J-5A</t>
-  </si>
-  <si>
-    <t>6A;6B;6C;6E;6O;6P;6Q;6W;6XC;6XF;6XH;8A</t>
-  </si>
-  <si>
-    <t>1B;6D;6G;6W;8A</t>
-  </si>
-  <si>
-    <t>6H</t>
-  </si>
-  <si>
-    <t>6H;8A</t>
-  </si>
-  <si>
-    <t>6L;6XJ</t>
-  </si>
-  <si>
-    <t>1A;1G;6H;6I;6L;6N;6W;6XE;6XG;6XJ;8A</t>
-  </si>
-  <si>
-    <t>1B;6O;6P;6W;6XF</t>
-  </si>
-  <si>
-    <t>6S</t>
-  </si>
-  <si>
-    <t>1J;6S</t>
-  </si>
-  <si>
-    <t>6G;6L;6N;6R;6W;6XA;6XD;6XG;6XH;8A;UNASSIGNED_1, 2J-5A</t>
-  </si>
-  <si>
-    <t>UNASSIGNED_1, 1B-1A</t>
-  </si>
-  <si>
-    <t>1A;1C</t>
-  </si>
-  <si>
-    <t>UNASSIGNED_1, 1C-1B</t>
-  </si>
-  <si>
-    <t>1A;1O</t>
+    <t>6C;6G;6H;6I;6L;6N;6Q;6R;6W;6XA;6XD;6XF;6XG;6XH;8A</t>
+  </si>
+  <si>
+    <t>1A;1D;UNASSIGNED_1, 1A-1B</t>
+  </si>
+  <si>
+    <t>1A;1B;1D;UNASSIGNED_1, 1B-1A</t>
   </si>
 </sst>
 </file>
@@ -958,7 +931,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1027,27 +1000,27 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
         <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
       <c r="C5" t="s">
         <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
@@ -1058,13 +1031,13 @@
         <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>24</v>
@@ -1126,98 +1099,98 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
         <v>33</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>39</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>40</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" t="s">
         <v>42</v>
-      </c>
-      <c r="B13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" t="s">
         <v>45</v>
-      </c>
-      <c r="B14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s">
         <v>47</v>
       </c>
-      <c r="B15" t="s">
-        <v>21</v>
-      </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
         <v>48</v>
@@ -1228,157 +1201,157 @@
         <v>49</v>
       </c>
       <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" t="s">
         <v>50</v>
-      </c>
-      <c r="C16" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" t="s">
         <v>52</v>
-      </c>
-      <c r="B17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" t="s">
         <v>54</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s">
         <v>56</v>
-      </c>
-      <c r="B19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D20" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D23" t="s">
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B25" t="s">
         <v>16</v>
@@ -1390,182 +1363,182 @@
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C26" t="s">
         <v>16</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D28" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C30" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="D31" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E31" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D32" t="s">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B33" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D33" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="E33" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="C34" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B35" t="s">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
         <v>16</v>
       </c>
       <c r="D35" t="s">
-        <v>16</v>
+        <v>90</v>
       </c>
       <c r="E35" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B36" t="s">
         <v>21</v>
@@ -1577,58 +1550,194 @@
         <v>16</v>
       </c>
       <c r="E36" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B37" t="s">
         <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E37" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B38" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C38" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E38" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
+        <v>99</v>
+      </c>
+      <c r="B39" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" t="s">
+        <v>16</v>
+      </c>
+      <c r="E40" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
         <v>102</v>
       </c>
-      <c r="B39" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" t="s">
-        <v>21</v>
-      </c>
-      <c r="D39" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" t="s">
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>104</v>
+      </c>
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>108</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" t="s">
+        <v>20</v>
+      </c>
+      <c r="E44" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>110</v>
+      </c>
+      <c r="B45" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" t="s">
+        <v>16</v>
+      </c>
+      <c r="E45" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>112</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E46" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>114</v>
+      </c>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" t="s">
+        <v>16</v>
+      </c>
+      <c r="D47" t="s">
+        <v>16</v>
+      </c>
+      <c r="E47" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1671,16 +1780,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1688,16 +1797,16 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>119</v>
       </c>
       <c r="E3" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1705,16 +1814,16 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
         <v>33</v>
       </c>
-      <c r="C4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
       <c r="E4" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1731,126 +1840,126 @@
         <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>123</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>128</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>116</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
         <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1858,174 +1967,174 @@
         <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E13" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>121</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>135</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>136</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>137</v>
       </c>
       <c r="E14" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>139</v>
       </c>
       <c r="B15" t="s">
-        <v>123</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>124</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>127</v>
+        <v>55</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E16" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
         <v>33</v>
       </c>
-      <c r="C17" t="s">
-        <v>17</v>
-      </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>143</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E18" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>131</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="E19" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="E20" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D22" t="s">
         <v>33</v>
       </c>
       <c r="E22" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="B23" t="s">
         <v>16</v>
@@ -2037,63 +2146,63 @@
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>139</v>
+        <v>17</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="D25" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>145</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>145</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B27" t="s">
         <v>21</v>
@@ -2105,80 +2214,80 @@
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>144</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D29" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="E29" t="s">
-        <v>79</v>
+        <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D30" t="s">
         <v>16</v>
       </c>
       <c r="E30" t="s">
-        <v>145</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C31" t="s">
-        <v>16</v>
+        <v>145</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>152</v>
       </c>
       <c r="E31" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="B32" t="s">
         <v>21</v>
@@ -2190,12 +2299,12 @@
         <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>148</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>149</v>
+        <v>94</v>
       </c>
       <c r="B33" t="s">
         <v>21</v>
@@ -2207,114 +2316,114 @@
         <v>16</v>
       </c>
       <c r="E33" t="s">
-        <v>150</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B34" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C34" t="s">
         <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>21</v>
       </c>
       <c r="C35" t="s">
-        <v>16</v>
+        <v>118</v>
       </c>
       <c r="D35" t="s">
-        <v>153</v>
+        <v>118</v>
       </c>
       <c r="E35" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B36" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>21</v>
+        <v>117</v>
       </c>
       <c r="D36" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E36" t="s">
-        <v>89</v>
+        <v>157</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B37" t="s">
-        <v>139</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="D37" t="s">
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="E37" t="s">
-        <v>155</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C38" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
       </c>
       <c r="E38" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>157</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
         <v>21</v>
       </c>
       <c r="C39" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D39" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
         <v>21</v>
@@ -2326,63 +2435,63 @@
         <v>16</v>
       </c>
       <c r="E40" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C41" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D41" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E41" t="s">
-        <v>159</v>
+        <v>109</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="B42" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C42" t="s">
-        <v>160</v>
+        <v>21</v>
       </c>
       <c r="D42" t="s">
-        <v>160</v>
+        <v>16</v>
       </c>
       <c r="E42" t="s">
-        <v>161</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B43" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C43" t="s">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="D43" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E43" t="s">
-        <v>162</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>163</v>
+        <v>114</v>
       </c>
       <c r="B44" t="s">
         <v>21</v>
@@ -2394,7 +2503,7 @@
         <v>16</v>
       </c>
       <c r="E44" t="s">
-        <v>164</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2405,7 +2514,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2437,16 +2546,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2454,16 +2563,16 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C3" t="s">
-        <v>167</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2474,13 +2583,13 @@
         <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2491,13 +2600,13 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2511,66 +2620,66 @@
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
         <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>7</v>
+        <v>152</v>
       </c>
       <c r="E8" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
@@ -2582,12 +2691,12 @@
         <v>16</v>
       </c>
       <c r="E10" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
@@ -2599,29 +2708,29 @@
         <v>16</v>
       </c>
       <c r="E11" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -2633,63 +2742,63 @@
         <v>16</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>175</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
       </c>
       <c r="E15" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -2701,131 +2810,131 @@
         <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>142</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D19" t="s">
-        <v>139</v>
+        <v>16</v>
       </c>
       <c r="E19" t="s">
-        <v>182</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>81</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>82</v>
+        <v>179</v>
       </c>
       <c r="B22" t="s">
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>153</v>
+        <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C23" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="D23" t="s">
-        <v>123</v>
+        <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>184</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>185</v>
+        <v>82</v>
       </c>
       <c r="B24" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D24" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="E24" t="s">
-        <v>186</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>151</v>
+        <v>86</v>
       </c>
       <c r="B25" t="s">
         <v>16</v>
@@ -2837,148 +2946,148 @@
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>187</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="C26" t="s">
-        <v>16</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="E26" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D27" t="s">
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="D28" t="s">
-        <v>166</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>188</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>93</v>
+        <v>182</v>
       </c>
       <c r="B29" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B30" t="s">
         <v>21</v>
       </c>
       <c r="C30" t="s">
-        <v>16</v>
+        <v>184</v>
       </c>
       <c r="D30" t="s">
-        <v>16</v>
+        <v>184</v>
       </c>
       <c r="E30" t="s">
-        <v>96</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>190</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C31" t="s">
         <v>21</v>
       </c>
       <c r="D31" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E31" t="s">
-        <v>191</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B32" t="s">
         <v>21</v>
       </c>
       <c r="C32" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="D32" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
       </c>
       <c r="E33" t="s">
-        <v>103</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>193</v>
+        <v>106</v>
       </c>
       <c r="B34" t="s">
         <v>21</v>
@@ -2990,24 +3099,75 @@
         <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>194</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>195</v>
+        <v>108</v>
       </c>
       <c r="B35" t="s">
         <v>21</v>
       </c>
       <c r="C35" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E35" t="s">
-        <v>196</v>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" t="s">
+        <v>16</v>
+      </c>
+      <c r="E36" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>114</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" t="s">
+        <v>16</v>
+      </c>
+      <c r="D38" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>